<commit_message>
Update Excel file 8/07/26
</commit_message>
<xml_diff>
--- a/12622743.xlsx
+++ b/12622743.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d41b41064dfff035/Desktop/pythonass/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="8_{ACC851C4-A9E2-44FB-A0C0-4C5573B75CE2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{18512A66-030D-48CC-98E5-F6DE9E17B26B}"/>
+  <xr:revisionPtr revIDLastSave="70" documentId="8_{ACC851C4-A9E2-44FB-A0C0-4C5573B75CE2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD89C775-2BAB-4917-B7A4-DD61081ACDDD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1390,47 +1390,91 @@
       <c r="N13" s="17"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46231</v>
+      </c>
+      <c r="B14" s="14">
+        <v>500</v>
+      </c>
+      <c r="C14" s="14">
+        <v>50</v>
+      </c>
+      <c r="D14" s="14">
+        <v>150</v>
+      </c>
+      <c r="E14" s="14">
+        <v>20</v>
+      </c>
+      <c r="F14" s="14">
+        <v>240</v>
+      </c>
+      <c r="G14" s="14">
+        <v>4</v>
+      </c>
+      <c r="H14" s="14">
+        <v>50</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
+        <v>430</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="N14" s="17"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="13">
+        <v>46232</v>
+      </c>
+      <c r="B15" s="14">
+        <v>550</v>
+      </c>
+      <c r="C15" s="14">
+        <v>240</v>
+      </c>
+      <c r="D15" s="14">
+        <v>180</v>
+      </c>
+      <c r="E15" s="14">
+        <v>80</v>
+      </c>
+      <c r="F15" s="14">
+        <v>0</v>
+      </c>
+      <c r="G15" s="14">
+        <v>0</v>
+      </c>
+      <c r="H15" s="14">
+        <v>90</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>1140</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
+        <v>300</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>61</v>
+      </c>
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Excel file 1/09/26
</commit_message>
<xml_diff>
--- a/12622743.xlsx
+++ b/12622743.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d41b41064dfff035/Desktop/pythonass/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="8_{ACC851C4-A9E2-44FB-A0C0-4C5573B75CE2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD89C775-2BAB-4917-B7A4-DD61081ACDDD}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="8_{ACC851C4-A9E2-44FB-A0C0-4C5573B75CE2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3779093-65A2-436B-B931-8226224F1A60}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -233,6 +233,9 @@
   </si>
   <si>
     <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Stressed</t>
   </si>
 </sst>
 </file>
@@ -1478,25 +1481,47 @@
       <c r="N15" s="17"/>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="A16" s="13">
+        <v>46233</v>
+      </c>
+      <c r="B16" s="14">
+        <v>450</v>
+      </c>
+      <c r="C16" s="14">
+        <v>180</v>
+      </c>
+      <c r="D16" s="14">
+        <v>420</v>
+      </c>
+      <c r="E16" s="14">
+        <v>55</v>
+      </c>
+      <c r="F16" s="14">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14">
+        <v>50</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>1155</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
+        <v>285</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update Excel file 3/09/26
</commit_message>
<xml_diff>
--- a/12622743.xlsx
+++ b/12622743.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d41b41064dfff035/Desktop/pythonass/CAP776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{ACC851C4-A9E2-44FB-A0C0-4C5573B75CE2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3779093-65A2-436B-B931-8226224F1A60}"/>
+  <xr:revisionPtr revIDLastSave="85" documentId="8_{ACC851C4-A9E2-44FB-A0C0-4C5573B75CE2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{286B2DE8-06AD-4D5D-9ABD-92BB8FDD7806}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="69">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Stressed</t>
+  </si>
+  <si>
+    <t>Excellent</t>
   </si>
 </sst>
 </file>
@@ -1086,7 +1089,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="18">
-        <v>46224</v>
+        <v>46255</v>
       </c>
       <c r="B7" s="19">
         <v>480</v>
@@ -1130,7 +1133,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="18">
-        <v>46225</v>
+        <v>46256</v>
       </c>
       <c r="B8" s="19">
         <v>660</v>
@@ -1174,7 +1177,7 @@
     </row>
     <row r="9" spans="1:14" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="18">
-        <v>46226</v>
+        <v>46257</v>
       </c>
       <c r="B9" s="19">
         <v>660</v>
@@ -1218,7 +1221,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="13">
-        <v>46227</v>
+        <v>46258</v>
       </c>
       <c r="B10" s="14">
         <v>500</v>
@@ -1262,7 +1265,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="13">
-        <v>46228</v>
+        <v>46259</v>
       </c>
       <c r="B11" s="14">
         <v>520</v>
@@ -1306,7 +1309,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
-        <v>46229</v>
+        <v>46260</v>
       </c>
       <c r="B12" s="14">
         <v>600</v>
@@ -1350,7 +1353,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="13">
-        <v>46230</v>
+        <v>46261</v>
       </c>
       <c r="B13" s="14">
         <v>560</v>
@@ -1394,7 +1397,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="13">
-        <v>46231</v>
+        <v>46262</v>
       </c>
       <c r="B14" s="14">
         <v>500</v>
@@ -1438,7 +1441,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="13">
-        <v>46232</v>
+        <v>46263</v>
       </c>
       <c r="B15" s="14">
         <v>550</v>
@@ -1482,7 +1485,7 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="13">
-        <v>46233</v>
+        <v>46264</v>
       </c>
       <c r="B16" s="14">
         <v>450</v>
@@ -1525,113 +1528,223 @@
       <c r="N16" s="17"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="A17" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B17" s="14">
+        <v>500</v>
+      </c>
+      <c r="C17" s="14">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14">
+        <v>320</v>
+      </c>
+      <c r="E17" s="14">
+        <v>50</v>
+      </c>
+      <c r="F17" s="14">
+        <v>240</v>
+      </c>
+      <c r="G17" s="14">
+        <v>4</v>
+      </c>
+      <c r="H17" s="14">
+        <v>0</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>1110</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
+        <v>330</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N17" s="17"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B18" s="14">
+        <v>550</v>
+      </c>
+      <c r="C18" s="14">
+        <v>0</v>
+      </c>
+      <c r="D18" s="14">
+        <v>60</v>
+      </c>
+      <c r="E18" s="14">
+        <v>10</v>
+      </c>
+      <c r="F18" s="14">
+        <v>420</v>
+      </c>
+      <c r="G18" s="14">
+        <v>7</v>
+      </c>
+      <c r="H18" s="14">
+        <v>0</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1040</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
+        <v>400</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>51</v>
+      </c>
       <c r="N18" s="17"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B19" s="14">
+        <v>420</v>
+      </c>
+      <c r="C19" s="14">
+        <v>50</v>
+      </c>
+      <c r="D19" s="14">
+        <v>80</v>
+      </c>
+      <c r="E19" s="14">
+        <v>20</v>
+      </c>
+      <c r="F19" s="14">
+        <v>50</v>
+      </c>
+      <c r="G19" s="14">
+        <v>1</v>
+      </c>
+      <c r="H19" s="14">
+        <v>180</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>800</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
+        <v>640</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="N19" s="17"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B20" s="14">
+        <v>560</v>
+      </c>
+      <c r="C20" s="14">
+        <v>100</v>
+      </c>
+      <c r="D20" s="14">
+        <v>0</v>
+      </c>
+      <c r="E20" s="14">
+        <v>50</v>
+      </c>
+      <c r="F20" s="14">
+        <v>240</v>
+      </c>
+      <c r="G20" s="14">
+        <v>4</v>
+      </c>
+      <c r="H20" s="14">
+        <v>0</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
+        <v>490</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="N20" s="17"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B21" s="14">
+        <v>500</v>
+      </c>
+      <c r="C21" s="14">
+        <v>50</v>
+      </c>
+      <c r="D21" s="14">
+        <v>180</v>
+      </c>
+      <c r="E21" s="14">
+        <v>120</v>
+      </c>
+      <c r="F21" s="14">
+        <v>300</v>
+      </c>
+      <c r="G21" s="14">
+        <v>5</v>
+      </c>
+      <c r="H21" s="14">
+        <v>0</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>1150</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
+        <v>290</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>65</v>
+      </c>
       <c r="N21" s="17"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">

</xml_diff>